<commit_message>
TAS DND changes Jan 22 2024
</commit_message>
<xml_diff>
--- a/TestData/TMTI0055011_VerifyInternalDealTeamSpecialtyRoleIncreasedLimitForFVALOBOpportunityEngagement.xlsx
+++ b/TestData/TMTI0055011_VerifyInternalDealTeamSpecialtyRoleIncreasedLimitForFVALOBOpportunityEngagement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812F5EB7-E21B-4C64-8022-0EE4EC519F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F12FEC-8F32-41F6-BE9B-AA88C33F7D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29010" windowHeight="14640" activeTab="3" xr2:uid="{4F41EB50-8C78-4F9F-A1D4-8B783E020697}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{4F41EB50-8C78-4F9F-A1D4-8B783E020697}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>

</xml_diff>